<commit_message>
Add Dr Yusuf Shittu to the partner tracker, with a conversation script
Met at the APPG on Black Maternal Health, 22 September 2026. A GP and
three-time founder on the NHS Clinical Entrepreneur Programme.

- Added to the partner CRM and target list as tier 2 clinical, priority
  8, stage 1 Identified. Only what was verifiable from a public profile
  is recorded; email and phone are marked not publicly available rather
  than guessed, and the LinkedIn slug is marked to confirm.
- New assets/CONVERSATION_YUSUF_SHITTU.md: opener, the one question that
  tests whether the record-keeping claim lands with clinicians, branches
  for either answer, what not to say, the same-evening message, and the
  months-long path from critic to clinical adviser.
- Counts updated from 74 to 75 partner organisations and contacts.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F19FGkn59tio4UCKXfsejn
</commit_message>
<xml_diff>
--- a/exports/xlsx/Partner_War_Room.xlsx
+++ b/exports/xlsx/Partner_War_Room.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 DASHBOARD" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 PARTNER CRM'!$A$1:$Z$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 TARGET LIST'!$A$1:$M$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01 PARTNER CRM'!$A$1:$Z$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02 TARGET LIST'!$A$1:$M$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -516,7 +516,7 @@
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>74 target organisations with the job title to approach, a CRM with the eleven-stage partner pipeline, stage rules and monthly KPIs.</t>
+          <t>75 target organisations and contacts with the job title to approach, a CRM with the eleven-stage partner pipeline, stage rules and monthly KPIs.</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z75"/>
+  <dimension ref="A1:Z76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7255,8 +7255,125 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Dr Yusuf Shittu — independent (NHS Clinical Entrepreneur Programme)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Clinician founder / adviser</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>2 Clinical</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Dr Yusuf Shittu</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>GP (MBBS MSc MRCGP); NHS Clinical Entrepreneur Programme; Imperial College London; healthcare designer and three-time founder</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com — profile confirmed, URL slug TO CONFIRM</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>EMAIL NOT PUBLICLY AVAILABLE</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>PHONE NOT PUBLICLY AVAILABLE</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Met in person</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Practising clinician who has built companies. Can say whether the record-keeping claim lands with clinicians or reads as admin. Knows the clinical safety officer market and the NHS innovation networks</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Honest product criticism; who should be the clinical safety officer; whether the Clinical Entrepreneur Programme has a route for a non-clinical founder; later, an introduction to a maternity clinician</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Nothing yet. Later: a named advisory role, paid, and equity if he takes it</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>22 Sep 2026 — APPG on Black Maternal Health, Committee Room 10</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Connect on LinkedIn same evening quoting something specific he said; then a 20-minute call</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>1 Identified</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>Met at the APPG. Do not ask him to be clinical safety officer yet — paid role with real liability. No email or phone held; do not guess one</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>Met in person at a public parliamentary event, 22 Sep 2026</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="X76" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="Y76" t="inlineStr">
+        <is>
+          <t>Adviser (unpaid first call)</t>
+        </is>
+      </c>
+      <c r="Z76" t="inlineStr">
+        <is>
+          <t>Met in person and exchanged details at a professional event — he can opt out at any time</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z75"/>
+  <autoFilter ref="A1:Z76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7267,7 +7384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11812,8 +11929,75 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Dr Yusuf Shittu — independent (NHS Clinical Entrepreneur Programme)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Clinician founder / adviser</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>2 Clinical</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>A GP who has founded three companies and sits inside the NHS Clinical Entrepreneur Programme. The fastest honest read on whether the product is useful to clinicians</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Twenty minutes of criticism; a view on the clinical safety officer; a view on the Clinical Entrepreneur route</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Nothing yet. A paid advisory role later if he is interested</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>N/A — approach him directly</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Adviser, then possible clinical advisory board</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Already met in person at the APPG on 22 Sep 2026. Follow up the same evening, referencing what he actually said</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Clinical credibility, safety officer route, and a door into the NHS innovation networks</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>LinkedIn profile seen 22 Sep 2026; no contact details held</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M75"/>
+  <autoFilter ref="A1:M76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>